<commit_message>
ban that toi 17/5/2026
</commit_message>
<xml_diff>
--- a/QuanLyKho/ContentBaoCaoXuatNhapTon.xlsx
+++ b/QuanLyKho/ContentBaoCaoXuatNhapTon.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <r xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <t xml:space="preserve">BỆNH VIỆN K
@@ -58,7 +58,7 @@
   </si>
   <si>
     <t xml:space="preserve">BẢNG TỔNG HỢP NHẬP - XUẤT - TỒN
-(Thời gian từ ngày 01/05/2026 đến ngày 13/05/2026)</t>
+(Thời gian từ ngày 01/05/2026 đến ngày 17/05/2026)</t>
   </si>
   <si>
     <t>STT</t>
@@ -79,16 +79,55 @@
     <t>Tồn cuối kỳ</t>
   </si>
   <si>
-    <t>1243435</t>
-  </si>
-  <si>
-    <t>Dây điện loại 1</t>
-  </si>
-  <si>
-    <t>Sản phẩm ABC</t>
-  </si>
-  <si>
-    <t>Sản phẩm B</t>
+    <t>Băng keo điện</t>
+  </si>
+  <si>
+    <t>Bóng đèn LED 12W</t>
+  </si>
+  <si>
+    <t>Bóng đèn LED 18W</t>
+  </si>
+  <si>
+    <t>Bút bi xanh</t>
+  </si>
+  <si>
+    <t>Cầu chì 10A</t>
+  </si>
+  <si>
+    <t>CB chống giật 30A</t>
+  </si>
+  <si>
+    <t>Công tắc đơn</t>
+  </si>
+  <si>
+    <t>Dây điện Cadivi 1.5mm</t>
+  </si>
+  <si>
+    <t>Dây điện Cadivi 2.5mm</t>
+  </si>
+  <si>
+    <t>Dây rút nhựa 20cm</t>
+  </si>
+  <si>
+    <t>Khăn lau công nghiệp</t>
+  </si>
+  <si>
+    <t>Kìm điện cách điện</t>
+  </si>
+  <si>
+    <t>Mũ bảo hộ</t>
+  </si>
+  <si>
+    <t>Ổ cắm điện 3 chấu</t>
+  </si>
+  <si>
+    <t>Ống nhựa PVC D21</t>
+  </si>
+  <si>
+    <t>Ống nhựa PVC D27</t>
+  </si>
+  <si>
+    <t>Tua vít 2 cạnh</t>
   </si>
   <si>
     <t>Tổng cộng</t>
@@ -634,7 +673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A22B4CD0-AB7D-4C47-8794-027CBD569E18}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" customWidth="1"/>
@@ -688,13 +727,13 @@
         <v>0</v>
       </c>
       <c r="D3" s="8">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="E3" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="7">
-        <v>0</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" ht="18.75" customHeight="1">
@@ -708,13 +747,13 @@
         <v>0</v>
       </c>
       <c r="D4" s="8">
-        <v>120</v>
+        <v>1</v>
       </c>
       <c r="E4" s="8">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F4" s="7">
-        <v>99</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="18.75" customHeight="1">
@@ -728,13 +767,13 @@
         <v>0</v>
       </c>
       <c r="D5" s="8">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E5" s="8">
         <v>0</v>
       </c>
       <c r="F5" s="7">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" ht="18.75" customHeight="1">
@@ -742,19 +781,19 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" s="7">
         <v>0</v>
       </c>
       <c r="D6" s="8">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E6" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F6" s="7">
-        <v>98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="18.75" customHeight="1">
@@ -762,141 +801,381 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="7">
+        <v>0</v>
+      </c>
+      <c r="D7" s="8">
+        <v>50</v>
+      </c>
+      <c r="E7" s="8">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" ht="18.75" customHeight="1">
+      <c r="A8" s="5">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0</v>
+      </c>
+      <c r="D8" s="8">
+        <v>0</v>
+      </c>
+      <c r="E8" s="8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="18.75" customHeight="1">
+      <c r="A9" s="5">
+        <v>7</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="7">
+        <v>0</v>
+      </c>
+      <c r="D9" s="8">
+        <v>0</v>
+      </c>
+      <c r="E9" s="8">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="18.75" customHeight="1">
+      <c r="A10" s="5">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="7">
+        <v>0</v>
+      </c>
+      <c r="D10" s="8">
+        <v>0</v>
+      </c>
+      <c r="E10" s="8">
+        <v>0</v>
+      </c>
+      <c r="F10" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="18.75" customHeight="1">
+      <c r="A11" s="5">
+        <v>9</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="7">
+        <v>0</v>
+      </c>
+      <c r="D11" s="8">
+        <v>0</v>
+      </c>
+      <c r="E11" s="8">
+        <v>0</v>
+      </c>
+      <c r="F11" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="18.75" customHeight="1">
+      <c r="A12" s="5">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="7">
+        <v>0</v>
+      </c>
+      <c r="D12" s="8">
+        <v>0</v>
+      </c>
+      <c r="E12" s="8">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="18.75" customHeight="1">
+      <c r="A13" s="5">
         <v>11</v>
       </c>
-      <c r="C7" s="7">
-        <v>0</v>
-      </c>
-      <c r="D7" s="8">
-        <v>200</v>
-      </c>
-      <c r="E7" s="8">
-        <v>1</v>
-      </c>
-      <c r="F7" s="7">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="7"/>
-    </row>
-    <row r="9" ht="37.5">
-      <c r="A9" s="5"/>
-      <c r="B9" s="9" t="s">
+      <c r="B13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="7">
+        <v>0</v>
+      </c>
+      <c r="D13" s="8">
+        <v>0</v>
+      </c>
+      <c r="E13" s="8">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="18.75" customHeight="1">
+      <c r="A14" s="5">
         <v>12</v>
       </c>
-      <c r="C9" s="10">
-        <f>SUM(C3:C8)</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="10">
-        <f>SUM(D3:D8)</f>
-        <v>0</v>
-      </c>
-      <c r="E9" s="10">
-        <f>SUM(E3:E8)</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="10">
-        <f>SUM(F3:F8)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" ht="18.75">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="13" t="s">
+      <c r="B14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="7">
+        <v>0</v>
+      </c>
+      <c r="D14" s="8">
+        <v>78176</v>
+      </c>
+      <c r="E14" s="8">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7">
+        <v>78176</v>
+      </c>
+    </row>
+    <row r="15" ht="18.75" customHeight="1">
+      <c r="A15" s="5">
         <v>13</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-    </row>
-    <row r="11" ht="18.75">
-      <c r="A11" s="14" t="s">
+      <c r="B15" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="7">
+        <v>0</v>
+      </c>
+      <c r="D15" s="8">
+        <v>0</v>
+      </c>
+      <c r="E15" s="8">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="18.75" customHeight="1">
+      <c r="A16" s="5">
         <v>14</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14" t="s">
+      <c r="B16" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="7">
+        <v>0</v>
+      </c>
+      <c r="D16" s="8">
+        <v>0</v>
+      </c>
+      <c r="E16" s="8">
+        <v>0</v>
+      </c>
+      <c r="F16" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="18.75" customHeight="1">
+      <c r="A17" s="5">
         <v>15</v>
       </c>
-      <c r="F11" s="14"/>
-    </row>
-    <row r="12" ht="18.75">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="16"/>
-    </row>
-    <row r="13" ht="18.75">
-      <c r="A13" s="16"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="16"/>
-    </row>
-    <row r="14" ht="18.75">
-      <c r="A14" s="16"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="16"/>
-    </row>
-    <row r="15" ht="18.75">
-      <c r="A15" s="16"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="16"/>
-    </row>
-    <row r="16" ht="18.75">
-      <c r="A16" s="16"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="16"/>
-    </row>
-    <row r="17" ht="18.75">
-      <c r="A17" s="16"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="16"/>
-    </row>
-    <row r="18" ht="18.75">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
+      <c r="B17" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="7">
+        <v>0</v>
+      </c>
+      <c r="D17" s="8">
+        <v>0</v>
+      </c>
+      <c r="E17" s="8">
+        <v>0</v>
+      </c>
+      <c r="F17" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="18.75" customHeight="1">
+      <c r="A18" s="5">
+        <v>16</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="7">
+        <v>0</v>
+      </c>
+      <c r="D18" s="8">
+        <v>0</v>
+      </c>
+      <c r="E18" s="8">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="18.75" customHeight="1">
+      <c r="A19" s="5">
+        <v>17</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="7">
+        <v>0</v>
+      </c>
+      <c r="D19" s="8">
+        <v>0</v>
+      </c>
+      <c r="E19" s="8">
+        <v>0</v>
+      </c>
+      <c r="F19" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="5"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" ht="37.5">
+      <c r="A21" s="5"/>
+      <c r="B21" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="10">
+        <f>SUM(C3:C20)</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="10">
+        <f>SUM(D3:D20)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="10">
+        <f>SUM(E3:E20)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="10">
+        <f>SUM(F3:F20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="18.75">
+      <c r="A22" s="11"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+    </row>
+    <row r="23" ht="18.75">
+      <c r="A23" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="14"/>
+    </row>
+    <row r="24" ht="18.75">
+      <c r="A24" s="15"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="16"/>
+    </row>
+    <row r="25" ht="18.75">
+      <c r="A25" s="16"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="16"/>
+    </row>
+    <row r="26" ht="18.75">
+      <c r="A26" s="16"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="16"/>
+    </row>
+    <row r="27" ht="18.75">
+      <c r="A27" s="16"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="16"/>
+    </row>
+    <row r="28" ht="18.75">
+      <c r="A28" s="16"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="16"/>
+    </row>
+    <row r="29" ht="18.75">
+      <c r="A29" s="16"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="16"/>
+    </row>
+    <row r="30" ht="18.75">
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
     </row>
   </sheetData>
   <mergeCells>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:F1"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>